<commit_message>
Add new build files for version 2.1.1 and update existing templates
</commit_message>
<xml_diff>
--- a/add_data/template_rdo.xlsx
+++ b/add_data/template_rdo.xlsx
@@ -63,7 +63,6 @@
         <sz val="10"/>
         <color theme="1"/>
         <rFont val="Calibri"/>
-        <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve">Consegna concessa </t>
     </r>
@@ -73,7 +72,6 @@
         <sz val="10"/>
         <color indexed="2"/>
         <rFont val="Calibri"/>
-        <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve">(in giorni lavorativi)</t>
     </r>
@@ -89,7 +87,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="6">
     <font>
       <sz val="11.000000"/>
       <color theme="1"/>
@@ -98,7 +96,6 @@
     </font>
     <font>
       <sz val="10.000000"/>
-      <color indexed="64"/>
       <name val="Calibri"/>
       <scheme val="minor"/>
     </font>
@@ -111,6 +108,7 @@
       <sz val="10.000000"/>
       <color indexed="2"/>
       <name val="Calibri"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <b/>
@@ -119,15 +117,9 @@
       <name val="Arial"/>
     </font>
     <font>
-      <sz val="10.000000"/>
-      <color indexed="64"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
       <b/>
       <sz val="10.000000"/>
       <name val="Calibri"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="3">
@@ -143,7 +135,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border>
       <left style="none"/>
       <right style="none"/>
@@ -161,7 +153,7 @@
       <top style="thin">
         <color auto="1"/>
       </top>
-      <bottom style="none"/>
+      <bottom/>
       <diagonal style="none"/>
     </border>
     <border>
@@ -179,11 +171,20 @@
       </bottom>
       <diagonal style="none"/>
     </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal style="none"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="17">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="1" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -204,25 +205,31 @@
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf fontId="1" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" shrinkToFit="1"/>
+    </xf>
+    <xf fontId="2" fillId="2" borderId="2" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf fontId="1" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" shrinkToFit="1"/>
-    </xf>
-    <xf fontId="5" fillId="2" borderId="2" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf fontId="1" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf fontId="6" fillId="0" borderId="2" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="1" fillId="0" borderId="3" numFmtId="164" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf fontId="1" fillId="0" borderId="3" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" shrinkToFit="1"/>
+    </xf>
+    <xf fontId="5" fillId="0" borderId="2" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf fontId="6" fillId="0" borderId="2" numFmtId="164" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="5" fillId="0" borderId="2" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" shrinkToFit="1" vertical="center" wrapText="1"/>
+    </xf>
+    <xf fontId="5" fillId="0" borderId="2" numFmtId="164" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf fontId="6" fillId="0" borderId="2" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" shrinkToFit="1" vertical="center" wrapText="1"/>
     </xf>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="164" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
@@ -727,9 +734,7 @@
     <col customWidth="1" min="1" max="2" width="20.7109375"/>
     <col customWidth="1" min="3" max="4" width="10.7109375"/>
     <col customWidth="1" min="5" max="5" width="40.7109375"/>
-    <col customWidth="1" min="6" max="7" width="20.7109375"/>
-    <col customWidth="1" min="8" max="8" width="40.7109375"/>
-    <col customWidth="1" min="9" max="12" width="10.7109375"/>
+    <col customWidth="1" min="6" max="9" width="10.7109375"/>
   </cols>
   <sheetData>
     <row r="1" ht="14.25">
@@ -748,64 +753,64 @@
       <c r="I1" s="7"/>
       <c r="J1" s="2"/>
       <c r="K1" s="2"/>
-      <c r="L1" s="8"/>
+      <c r="L1" s="7"/>
     </row>
     <row r="2" ht="14.25">
       <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
       <c r="B2" s="2"/>
-      <c r="C2" s="9"/>
+      <c r="C2" s="8"/>
       <c r="D2" s="1"/>
-      <c r="E2" s="7"/>
-      <c r="F2" s="7"/>
-      <c r="G2" s="7"/>
+      <c r="E2" s="9"/>
+      <c r="F2" s="9"/>
+      <c r="G2" s="9"/>
       <c r="H2" s="10"/>
       <c r="I2" s="7"/>
-      <c r="J2" s="2"/>
-      <c r="K2" s="2"/>
-      <c r="L2" s="8"/>
+      <c r="J2" s="11"/>
+      <c r="K2" s="11"/>
+      <c r="L2" s="12"/>
     </row>
     <row r="3" ht="54">
-      <c r="A3" s="11" t="s">
+      <c r="A3" s="13" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="11" t="s">
+      <c r="B3" s="13" t="s">
         <v>4</v>
       </c>
-      <c r="C3" s="11" t="s">
+      <c r="C3" s="13" t="s">
         <v>5</v>
       </c>
-      <c r="D3" s="11" t="s">
+      <c r="D3" s="13" t="s">
         <v>6</v>
       </c>
-      <c r="E3" s="11" t="s">
+      <c r="E3" s="13" t="s">
         <v>7</v>
       </c>
-      <c r="F3" s="11" t="s">
+      <c r="F3" s="13" t="s">
         <v>8</v>
       </c>
-      <c r="G3" s="11" t="s">
+      <c r="G3" s="13" t="s">
         <v>9</v>
       </c>
-      <c r="H3" s="11" t="s">
+      <c r="H3" s="13" t="s">
         <v>10</v>
       </c>
-      <c r="I3" s="11" t="s">
+      <c r="I3" s="14" t="s">
         <v>11</v>
       </c>
-      <c r="J3" s="12" t="s">
+      <c r="J3" s="15" t="s">
         <v>12</v>
       </c>
-      <c r="K3" s="12" t="s">
+      <c r="K3" s="15" t="s">
         <v>13</v>
       </c>
-      <c r="L3" s="13" t="s">
+      <c r="L3" s="14" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="4" ht="14.25">
-      <c r="J4" s="14"/>
+      <c r="G4" s="16"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>